<commit_message>
provenance as link, not as card
</commit_message>
<xml_diff>
--- a/misc/customizing-labels.xlsx
+++ b/misc/customizing-labels.xlsx
@@ -9,7 +9,7 @@
     <sheet name="rowsForView" r:id="rId3" sheetId="1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">rowsForView!$A$1:$F$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">rowsForView!$A$1:$F$116</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -383,26 +383,26 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>eth.illLink.text1</t>
+          <t>slsp.getit.reservationText</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>Article/chapter is not held in the swisscovery Network or cannot be requested from a library at ETH Zurich.</t>
+          <t>Reserve</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Artikel/Kapitel ist im swisscovery Netzwerk nicht vorhanden oder  nicht an eine Bibliothek der ETH Zürich bestellbar. </t>
+          <t>Reservieren</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>bernd.uttenweiler@library.ethz.ch</t>
+          <t>Network</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>46255.0</v>
+        <v>46286.0</v>
       </c>
     </row>
     <row r="11">
@@ -413,17 +413,17 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>eth.illLink.text2</t>
+          <t>eth.illLink.text1</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>Please request via</t>
+          <t>Article/chapter is not held in the swisscovery Network or cannot be requested from a library at ETH Zurich.</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>Bestellen Sie bitte via</t>
+          <t xml:space="preserve">Artikel/Kapitel ist im swisscovery Netzwerk nicht vorhanden oder  nicht an eine Bibliothek der ETH Zürich bestellbar. </t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr">
@@ -432,7 +432,7 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>46058.0</v>
+        <v>46255.0</v>
       </c>
     </row>
     <row r="12">
@@ -443,17 +443,17 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>eth.illLink.text3</t>
+          <t>eth.illLink.text2</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>Please request via</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>Bestellen Sie bitte via</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
@@ -473,17 +473,17 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>eth.illLink.linkText</t>
+          <t>eth.illLink.text3</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>interlibrary loan</t>
+          <t>.</t>
         </is>
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>Fernleihe</t>
+          <t>.</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr">
@@ -503,17 +503,17 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>eth.illLink.url</t>
+          <t>eth.illLink.linkText</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>https://library.ethz.ch/en/find-media/borrowing-and-using/order-forms/interlibrary-loans-ordering-copies.html</t>
+          <t>interlibrary loan</t>
         </is>
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>https://library.ethz.ch/medien-finden/ausleihen-und-nutzen/bestellformulare/fernleihe-kopien-bestellen.html</t>
+          <t>Fernleihe</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>46097.0</v>
+        <v>46058.0</v>
       </c>
     </row>
     <row r="15">
@@ -533,17 +533,17 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>eth.composeErara.print</t>
+          <t>eth.illLink.url</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>Print item in ETH swisscovery</t>
+          <t>https://library.ethz.ch/en/find-media/borrowing-and-using/order-forms/interlibrary-loans-ordering-copies.html</t>
         </is>
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>Print-Exemplar in ETH swisscovery</t>
+          <t>https://library.ethz.ch/medien-finden/ausleihen-und-nutzen/bestellformulare/fernleihe-kopien-bestellen.html</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr">
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>46058.0</v>
+        <v>46097.0</v>
       </c>
     </row>
     <row r="16">
@@ -563,17 +563,17 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>eth.composeErara.online</t>
+          <t>eth.composeErara.print</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>Online item in ETH swisscovery (from e-rara)</t>
+          <t>Print item in ETH swisscovery</t>
         </is>
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>Online-Exemplar in ETH swisscovery (e-rara)</t>
+          <t>Print-Exemplar in ETH swisscovery</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr">
@@ -593,17 +593,17 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>eth.composeErara.emaps</t>
+          <t>eth.composeErara.online</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>Georeferenced online item in ETH swisscovery (from e-maps)</t>
+          <t>Online item in ETH swisscovery (from e-rara)</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>Georeferenziertes Online-Exemplar in ETH swisscovery (e-maps)</t>
+          <t>Online-Exemplar in ETH swisscovery (e-rara)</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr">
@@ -623,17 +623,17 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>eth.composeErara.geoTiff</t>
+          <t>eth.composeErara.emaps</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>GeoTIFF map via e-maps</t>
+          <t>Georeferenced online item in ETH swisscovery (from e-maps)</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
         <is>
-          <t>GeoTIFF via e-maps</t>
+          <t>Georeferenziertes Online-Exemplar in ETH swisscovery (e-maps)</t>
         </is>
       </c>
       <c r="E18" s="1" t="inlineStr">
@@ -653,17 +653,17 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>eth.composeNb.print</t>
+          <t>eth.composeErara.geoTiff</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>Print item in in ETH swisscovery</t>
+          <t>GeoTIFF map via e-maps</t>
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr">
         <is>
-          <t>Print-Exemplar in ETH swisscovery</t>
+          <t>GeoTIFF via e-maps</t>
         </is>
       </c>
       <c r="E19" s="1" t="inlineStr">
@@ -683,17 +683,17 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>eth.composeNb.online</t>
+          <t>eth.composeNb.print</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>Online item in ETH swisscovery</t>
+          <t>Print item in in ETH swisscovery</t>
         </is>
       </c>
       <c r="D20" s="1" t="inlineStr">
         <is>
-          <t>Online-Exemplar in ETH swisscovery</t>
+          <t>Print-Exemplar in ETH swisscovery</t>
         </is>
       </c>
       <c r="E20" s="1" t="inlineStr">
@@ -713,17 +713,17 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>eth.dnbToc.toc</t>
+          <t>eth.composeNb.online</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>Table of content from the DNB for</t>
+          <t>Online item in ETH swisscovery</t>
         </is>
       </c>
       <c r="D21" s="1" t="inlineStr">
         <is>
-          <t>Inhaltsverzeichnis der DNB zu</t>
+          <t>Online-Exemplar in ETH swisscovery</t>
         </is>
       </c>
       <c r="E21" s="1" t="inlineStr">
@@ -743,17 +743,17 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>eth.dnbToc.text</t>
+          <t>eth.dnbToc.toc</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>Content description from the DNB for</t>
+          <t>Table of content from the DNB for</t>
         </is>
       </c>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t>Inhaltstext der DNB zu</t>
+          <t>Inhaltsverzeichnis der DNB zu</t>
         </is>
       </c>
       <c r="E22" s="1" t="inlineStr">
@@ -773,17 +773,17 @@
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>eth.libraryStack.text1</t>
+          <t>eth.dnbToc.text</t>
         </is>
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>Password protected access. Restricted to members of ETH Zurich only.</t>
+          <t>Content description from the DNB for</t>
         </is>
       </c>
       <c r="D23" s="1" t="inlineStr">
         <is>
-          <t>Passwortgeschützter Zugang. Nur für Mitglieder der ETH Zürich zugänglich.</t>
+          <t>Inhaltstext der DNB zu</t>
         </is>
       </c>
       <c r="E23" s="1" t="inlineStr">
@@ -803,17 +803,17 @@
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>eth.libraryStack.text2</t>
+          <t>eth.libraryStack.text1</t>
         </is>
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>You need to register with your ETH Zurich e-mail address "Sign In". Access to this source is restricted on the domain ethz.ch because of license restrictions.</t>
+          <t>Password protected access. Restricted to members of ETH Zurich only.</t>
         </is>
       </c>
       <c r="D24" s="1" t="inlineStr">
         <is>
-          <t>Sie müssen sich mit Ihrer ETH Zürich E-Mail-Adresse unter „Anmelden” registrieren. Der Zugriff auf diese Quelle ist aufgrund von Lizenzbeschränkungen auf die Domain ethz.ch eingeschränkt.</t>
+          <t>Passwortgeschützter Zugang. Nur für Mitglieder der ETH Zürich zugänglich.</t>
         </is>
       </c>
       <c r="E24" s="1" t="inlineStr">
@@ -833,17 +833,17 @@
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>eth.wayback.text</t>
+          <t>eth.libraryStack.text2</t>
         </is>
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t>In the web archive, select a year and a date marked in blue to access the archived website.</t>
+          <t>You need to register with your ETH Zurich e-mail address "Sign In". Access to this source is restricted on the domain ethz.ch because of license restrictions.</t>
         </is>
       </c>
       <c r="D25" s="1" t="inlineStr">
         <is>
-          <t>Wählen Sie im Webarchiv ein Jahr und ein blau markiertes Datum, um die archivierte Website aufzurufen.</t>
+          <t>Sie müssen sich mit Ihrer ETH Zürich E-Mail-Adresse unter „Anmelden” registrieren. Der Zugriff auf diese Quelle ist aufgrund von Lizenzbeschränkungen auf die Domain ethz.ch eingeschränkt.</t>
         </is>
       </c>
       <c r="E25" s="1" t="inlineStr">
@@ -863,17 +863,17 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>eth.wayback.linkText</t>
+          <t>eth.wayback.text</t>
         </is>
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>Link to the web archive</t>
+          <t>In the web archive, select a year and a date marked in blue to access the archived website.</t>
         </is>
       </c>
       <c r="D26" s="1" t="inlineStr">
         <is>
-          <t>Link zum Webarchiv</t>
+          <t>Wählen Sie im Webarchiv ein Jahr und ein blau markiertes Datum, um die archivierte Website aufzurufen.</t>
         </is>
       </c>
       <c r="E26" s="1" t="inlineStr">
@@ -893,17 +893,17 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>eth.onlineProblem.linkText</t>
+          <t>eth.wayback.linkText</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>Report access problem</t>
+          <t>Link to the web archive</t>
         </is>
       </c>
       <c r="D27" s="1" t="inlineStr">
         <is>
-          <t>Zugriffsproblem melden</t>
+          <t>Link zum Webarchiv</t>
         </is>
       </c>
       <c r="E27" s="1" t="inlineStr">
@@ -923,17 +923,17 @@
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>eth.onlineProblem.ariaLabel</t>
+          <t>eth.onlineProblem.linkText</t>
         </is>
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>Report access problem by email</t>
+          <t>Report access problem</t>
         </is>
       </c>
       <c r="D28" s="1" t="inlineStr">
         <is>
-          <t>Zugriffsproblem per E-Mail melden</t>
+          <t>Zugriffsproblem melden</t>
         </is>
       </c>
       <c r="E28" s="1" t="inlineStr">
@@ -953,17 +953,17 @@
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>eth.registrationLink.linkText</t>
+          <t>eth.onlineProblem.ariaLabel</t>
         </is>
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t>Not registered yet?</t>
+          <t>Report access problem by email</t>
         </is>
       </c>
       <c r="D29" s="1" t="inlineStr">
         <is>
-          <t>Noch nicht registriert?</t>
+          <t>Zugriffsproblem per E-Mail melden</t>
         </is>
       </c>
       <c r="E29" s="1" t="inlineStr">
@@ -983,17 +983,17 @@
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>eth.onlineButton.linkText</t>
+          <t>eth.registrationLink.linkText</t>
         </is>
       </c>
       <c r="C30" s="1" t="inlineStr">
         <is>
-          <t>View Online</t>
+          <t>Not registered yet?</t>
         </is>
       </c>
       <c r="D30" s="1" t="inlineStr">
         <is>
-          <t>Online ansehen</t>
+          <t>Noch nicht registriert?</t>
         </is>
       </c>
       <c r="E30" s="1" t="inlineStr">
@@ -1013,17 +1013,17 @@
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>eth.okm.label</t>
+          <t>eth.onlineButton.linkText</t>
         </is>
       </c>
       <c r="C31" s="1" t="inlineStr">
         <is>
-          <t>Search for “{{ search }}” in Open Knowledge Maps:</t>
+          <t>View Online</t>
         </is>
       </c>
       <c r="D31" s="1" t="inlineStr">
         <is>
-          <t>Suche nach “{{ search }}” in Open Knowledge Maps:</t>
+          <t>Online ansehen</t>
         </is>
       </c>
       <c r="E31" s="1" t="inlineStr">
@@ -1043,17 +1043,17 @@
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>eth.logoSubline.subline</t>
+          <t>eth.okm.label</t>
         </is>
       </c>
       <c r="C32" s="1" t="inlineStr">
         <is>
-          <t>ETH swisscovery</t>
+          <t>Search for “{{ search }}” in Open Knowledge Maps:</t>
         </is>
       </c>
       <c r="D32" s="1" t="inlineStr">
         <is>
-          <t>ETH swisscovery</t>
+          <t>Suche nach “{{ search }}” in Open Knowledge Maps:</t>
         </is>
       </c>
       <c r="E32" s="1" t="inlineStr">
@@ -1073,17 +1073,17 @@
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>eth.idpWarning.text1</t>
+          <t>eth.logoSubline.subline</t>
         </is>
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t>Link your SWICTH edu-ID to your ETH Zurich user account in</t>
+          <t>ETH swisscovery</t>
         </is>
       </c>
       <c r="D33" s="1" t="inlineStr">
         <is>
-          <t>Verknüpfen Sie Ihre SWITCH edu-ID mit Ihrem ETH-Benutzerkonto in</t>
+          <t>ETH swisscovery</t>
         </is>
       </c>
       <c r="E33" s="1" t="inlineStr">
@@ -1103,17 +1103,17 @@
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>eth.idpWarning.text2</t>
+          <t>eth.idpWarning.text1</t>
         </is>
       </c>
       <c r="C34" s="1" t="inlineStr">
         <is>
-          <t>to benefit from the advantages for members of ETH Zurich.</t>
+          <t>Link your SWICTH edu-ID to your ETH Zurich user account in</t>
         </is>
       </c>
       <c r="D34" s="1" t="inlineStr">
         <is>
-          <t>, um von den Vorteilen für ETH-Angehörige zu profitieren.</t>
+          <t>Verknüpfen Sie Ihre SWITCH edu-ID mit Ihrem ETH-Benutzerkonto in</t>
         </is>
       </c>
       <c r="E34" s="1" t="inlineStr">
@@ -1133,17 +1133,17 @@
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>eth.idpWarning.linkText2</t>
+          <t>eth.idpWarning.text2</t>
         </is>
       </c>
       <c r="C35" s="1" t="inlineStr">
         <is>
-          <t>Instructions</t>
+          <t>to benefit from the advantages for members of ETH Zurich.</t>
         </is>
       </c>
       <c r="D35" s="1" t="inlineStr">
         <is>
-          <t>Anleitung</t>
+          <t>, um von den Vorteilen für ETH-Angehörige zu profitieren.</t>
         </is>
       </c>
       <c r="E35" s="1" t="inlineStr">
@@ -1163,17 +1163,17 @@
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>eth.idpWarning.linkText1</t>
+          <t>eth.idpWarning.linkText2</t>
         </is>
       </c>
       <c r="C36" s="1" t="inlineStr">
         <is>
-          <t>https://www.password.ethz.ch/</t>
+          <t>Instructions</t>
         </is>
       </c>
       <c r="D36" s="1" t="inlineStr">
         <is>
-          <t>https://www.password.ethz.ch/</t>
+          <t>Anleitung</t>
         </is>
       </c>
       <c r="E36" s="1" t="inlineStr">
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>46260.0</v>
+        <v>46058.0</v>
       </c>
     </row>
     <row r="37">
@@ -1193,17 +1193,17 @@
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>eth.idpWarning.link1</t>
+          <t>eth.idpWarning.linkText1</t>
         </is>
       </c>
       <c r="C37" s="1" t="inlineStr">
         <is>
-          <t>https://www.password.ethz.ch/authentication/login_en.html</t>
+          <t>https://www.password.ethz.ch/</t>
         </is>
       </c>
       <c r="D37" s="1" t="inlineStr">
         <is>
-          <t>https://www.password.ethz.ch/authentication/login.html</t>
+          <t>https://www.password.ethz.ch/</t>
         </is>
       </c>
       <c r="E37" s="1" t="inlineStr">
@@ -1223,17 +1223,17 @@
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>eth.idpWarning.link2</t>
+          <t>eth.idpWarning.link1</t>
         </is>
       </c>
       <c r="C38" s="1" t="inlineStr">
         <is>
-          <t>https://library.ethz.ch/en/find-media/borrowing-and-using/frequently-asked-questions.html#eth-card-as-user-id</t>
+          <t>https://www.password.ethz.ch/authentication/login_en.html</t>
         </is>
       </c>
       <c r="D38" s="1" t="inlineStr">
         <is>
-          <t>https://library.ethz.ch/medien-finden/ausleihen-und-nutzen/faq.html#eth-karte-als-benutzungsausweis</t>
+          <t>https://www.password.ethz.ch/authentication/login.html</t>
         </is>
       </c>
       <c r="E38" s="1" t="inlineStr">
@@ -1242,7 +1242,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>46163.0</v>
+        <v>46260.0</v>
       </c>
     </row>
     <row r="39">
@@ -1253,17 +1253,17 @@
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>eth.changeAddress.heading</t>
+          <t>eth.idpWarning.link2</t>
         </is>
       </c>
       <c r="C39" s="1" t="inlineStr">
         <is>
-          <t>Address changes</t>
+          <t>https://library.ethz.ch/en/find-media/borrowing-and-using/frequently-asked-questions.html#eth-card-as-user-id</t>
         </is>
       </c>
       <c r="D39" s="1" t="inlineStr">
         <is>
-          <t>Adresse bearbeiten</t>
+          <t>https://library.ethz.ch/medien-finden/ausleihen-und-nutzen/faq.html#eth-karte-als-benutzungsausweis</t>
         </is>
       </c>
       <c r="E39" s="1" t="inlineStr">
@@ -1272,7 +1272,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>46058.0</v>
+        <v>46163.0</v>
       </c>
     </row>
     <row r="40">
@@ -1283,17 +1283,17 @@
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t>eth.changeAddress.ethMembers</t>
+          <t>eth.changeAddress.heading</t>
         </is>
       </c>
       <c r="C40" s="1" t="inlineStr">
         <is>
-          <t>Members of ETH</t>
+          <t>Address changes</t>
         </is>
       </c>
       <c r="D40" s="1" t="inlineStr">
         <is>
-          <t>ETH-Angehörige</t>
+          <t>Adresse bearbeiten</t>
         </is>
       </c>
       <c r="E40" s="1" t="inlineStr">
@@ -1313,17 +1313,17 @@
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>eth.changeAddress.ethMembersIntro</t>
+          <t>eth.changeAddress.ethMembers</t>
         </is>
       </c>
       <c r="C41" s="1" t="inlineStr">
         <is>
-          <t>Change your address in 2 steps:</t>
+          <t>Members of ETH</t>
         </is>
       </c>
       <c r="D41" s="1" t="inlineStr">
         <is>
-          <t>Ändern Sie Ihre Adresse in 2 Schritten:</t>
+          <t>ETH-Angehörige</t>
         </is>
       </c>
       <c r="E41" s="1" t="inlineStr">
@@ -1343,17 +1343,17 @@
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
-          <t>eth.changeAddress.ethMembersStep1</t>
+          <t>eth.changeAddress.ethMembersIntro</t>
         </is>
       </c>
       <c r="C42" s="1" t="inlineStr">
         <is>
-          <t>1. Change address:</t>
+          <t>Change your address in 2 steps:</t>
         </is>
       </c>
       <c r="D42" s="1" t="inlineStr">
         <is>
-          <t>1. Adresse ändern:</t>
+          <t>Ändern Sie Ihre Adresse in 2 Schritten:</t>
         </is>
       </c>
       <c r="E42" s="1" t="inlineStr">
@@ -1373,17 +1373,17 @@
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t>eth.changeAddress.ethMembersStep2</t>
+          <t>eth.changeAddress.ethMembersStep1</t>
         </is>
       </c>
       <c r="C43" s="1" t="inlineStr">
         <is>
-          <t>2. Confirm address change:</t>
+          <t>1. Change address:</t>
         </is>
       </c>
       <c r="D43" s="1" t="inlineStr">
         <is>
-          <t>2. Adressänderung bestätigen:</t>
+          <t>1. Adresse ändern:</t>
         </is>
       </c>
       <c r="E43" s="1" t="inlineStr">
@@ -1403,17 +1403,17 @@
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>eth.changeAddress.otherCustomers</t>
+          <t>eth.changeAddress.ethMembersStep2</t>
         </is>
       </c>
       <c r="C44" s="1" t="inlineStr">
         <is>
-          <t>Private individuals</t>
+          <t>2. Confirm address change:</t>
         </is>
       </c>
       <c r="D44" s="1" t="inlineStr">
         <is>
-          <t>Privatpersonen</t>
+          <t>2. Adressänderung bestätigen:</t>
         </is>
       </c>
       <c r="E44" s="1" t="inlineStr">
@@ -1433,17 +1433,17 @@
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>eth.changeAddress.otherCustomersIntro</t>
+          <t>eth.changeAddress.otherCustomers</t>
         </is>
       </c>
       <c r="C45" s="1" t="inlineStr">
         <is>
-          <t>Change your address here:</t>
+          <t>Private individuals</t>
         </is>
       </c>
       <c r="D45" s="1" t="inlineStr">
         <is>
-          <t>Ändern Sie Ihre Adresse hier:</t>
+          <t>Privatpersonen</t>
         </is>
       </c>
       <c r="E45" s="1" t="inlineStr">
@@ -1463,17 +1463,17 @@
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>eth.changeAddress.ethMembersStep1Url</t>
+          <t>eth.changeAddress.otherCustomersIntro</t>
         </is>
       </c>
       <c r="C46" s="1" t="inlineStr">
         <is>
-          <t>https://idapps.ethz.ch/contact-data/</t>
+          <t>Change your address here:</t>
         </is>
       </c>
       <c r="D46" s="1" t="inlineStr">
         <is>
-          <t>https://idapps.ethz.ch/contact-data/</t>
+          <t>Ändern Sie Ihre Adresse hier:</t>
         </is>
       </c>
       <c r="E46" s="1" t="inlineStr">
@@ -1482,7 +1482,7 @@
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>46141.0</v>
+        <v>46058.0</v>
       </c>
     </row>
     <row r="47">
@@ -1493,17 +1493,17 @@
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>eth.changeAddress.ethMembersStep2Url</t>
+          <t>eth.changeAddress.ethMembersStep1Url</t>
         </is>
       </c>
       <c r="C47" s="1" t="inlineStr">
         <is>
-          <t>https://eduid.ch</t>
+          <t>https://idapps.ethz.ch/contact-data/</t>
         </is>
       </c>
       <c r="D47" s="1" t="inlineStr">
         <is>
-          <t>https://eduid.ch</t>
+          <t>https://idapps.ethz.ch/contact-data/</t>
         </is>
       </c>
       <c r="E47" s="1" t="inlineStr">
@@ -1512,7 +1512,7 @@
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>46058.0</v>
+        <v>46141.0</v>
       </c>
     </row>
     <row r="48">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t>eth.changeAddress.otherCustomersUrl</t>
+          <t>eth.changeAddress.ethMembersStep2Url</t>
         </is>
       </c>
       <c r="C48" s="1" t="inlineStr">
@@ -1553,17 +1553,17 @@
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t>eth.bibNews.all</t>
+          <t>eth.changeAddress.otherCustomersUrl</t>
         </is>
       </c>
       <c r="C49" s="1" t="inlineStr">
         <is>
-          <t>All news</t>
+          <t>https://eduid.ch</t>
         </is>
       </c>
       <c r="D49" s="1" t="inlineStr">
         <is>
-          <t>Alle News</t>
+          <t>https://eduid.ch</t>
         </is>
       </c>
       <c r="E49" s="1" t="inlineStr">
@@ -1583,17 +1583,17 @@
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t>eth.geoRef.heading</t>
+          <t>eth.bibNews.all</t>
         </is>
       </c>
       <c r="C50" s="1" t="inlineStr">
         <is>
-          <t>Related Places</t>
+          <t>All news</t>
         </is>
       </c>
       <c r="D50" s="1" t="inlineStr">
         <is>
-          <t>Verknüpfte Orte</t>
+          <t>Alle News</t>
         </is>
       </c>
       <c r="E50" s="1" t="inlineStr">
@@ -1613,17 +1613,17 @@
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>eth.geoRef.entity</t>
+          <t>eth.geoRef.heading</t>
         </is>
       </c>
       <c r="C51" s="1" t="inlineStr">
         <is>
-          <t>Place</t>
+          <t>Related Places</t>
         </is>
       </c>
       <c r="D51" s="1" t="inlineStr">
         <is>
-          <t>Ort</t>
+          <t>Verknüpfte Orte</t>
         </is>
       </c>
       <c r="E51" s="1" t="inlineStr">
@@ -1643,17 +1643,17 @@
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t>eth.provenance.heading</t>
+          <t>eth.geoRef.entity</t>
         </is>
       </c>
       <c r="C52" s="1" t="inlineStr">
         <is>
-          <t>Provenance marks</t>
+          <t>Place</t>
         </is>
       </c>
       <c r="D52" s="1" t="inlineStr">
         <is>
-          <t>Provenienzen</t>
+          <t>Ort</t>
         </is>
       </c>
       <c r="E52" s="1" t="inlineStr">
@@ -1673,17 +1673,17 @@
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t>eth.provenance.entity</t>
+          <t>eth.provenance.heading</t>
         </is>
       </c>
       <c r="C53" s="1" t="inlineStr">
         <is>
-          <t>Provenance</t>
+          <t>Provenance marks</t>
         </is>
       </c>
       <c r="D53" s="1" t="inlineStr">
         <is>
-          <t>Provenienz</t>
+          <t>Provenienzen</t>
         </is>
       </c>
       <c r="E53" s="1" t="inlineStr">
@@ -1703,17 +1703,17 @@
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
-          <t>eth.provenance.date</t>
+          <t>eth.provenance.entity</t>
         </is>
       </c>
       <c r="C54" s="1" t="inlineStr">
         <is>
-          <t>Date:</t>
+          <t>Provenance</t>
         </is>
       </c>
       <c r="D54" s="1" t="inlineStr">
         <is>
-          <t>Datierung:</t>
+          <t>Provenienz</t>
         </is>
       </c>
       <c r="E54" s="1" t="inlineStr">
@@ -1733,17 +1733,17 @@
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
-          <t>eth.provenance.epicsLinkText</t>
+          <t>eth.provenance.date</t>
         </is>
       </c>
       <c r="C55" s="1" t="inlineStr">
         <is>
-          <t>Provenance in E-Pics</t>
+          <t>Date:</t>
         </is>
       </c>
       <c r="D55" s="1" t="inlineStr">
         <is>
-          <t>Provenienz in E-Pics</t>
+          <t>Datierung:</t>
         </is>
       </c>
       <c r="E55" s="1" t="inlineStr">
@@ -1763,17 +1763,17 @@
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
-          <t>eth.personCard.entity</t>
+          <t>eth.provenance.epicsLinkText</t>
         </is>
       </c>
       <c r="C56" s="1" t="inlineStr">
         <is>
-          <t>Person</t>
+          <t>Provenance in E-Pics</t>
         </is>
       </c>
       <c r="D56" s="1" t="inlineStr">
         <is>
-          <t>Person</t>
+          <t>Provenienz in E-Pics</t>
         </is>
       </c>
       <c r="E56" s="1" t="inlineStr">
@@ -1793,17 +1793,17 @@
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
-          <t>eth.personCard.photo</t>
+          <t>eth.personCard.entity</t>
         </is>
       </c>
       <c r="C57" s="1" t="inlineStr">
         <is>
-          <t>Photo of</t>
+          <t>Person</t>
         </is>
       </c>
       <c r="D57" s="1" t="inlineStr">
         <is>
-          <t>Photo von</t>
+          <t>Person</t>
         </is>
       </c>
       <c r="E57" s="1" t="inlineStr">
@@ -1823,17 +1823,17 @@
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
-          <t>eth.personCard.licence</t>
+          <t>eth.personCard.photo</t>
         </is>
       </c>
       <c r="C58" s="1" t="inlineStr">
         <is>
-          <t>Licence for the picture see</t>
+          <t>Photo of</t>
         </is>
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>Lizenz für das Bild siehe</t>
+          <t>Photo von</t>
         </is>
       </c>
       <c r="E58" s="1" t="inlineStr">
@@ -1853,17 +1853,17 @@
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
-          <t>eth.personCard.heading</t>
+          <t>eth.personCard.licence</t>
         </is>
       </c>
       <c r="C59" s="1" t="inlineStr">
         <is>
-          <t>Related Persons</t>
+          <t>Licence for the picture see</t>
         </is>
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>Verknüpfte Personen</t>
+          <t>Lizenz für das Bild siehe</t>
         </is>
       </c>
       <c r="E59" s="1" t="inlineStr">
@@ -1883,17 +1883,17 @@
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
-          <t>eth.personCard.headingMore</t>
+          <t>eth.personCard.heading</t>
         </is>
       </c>
       <c r="C60" s="1" t="inlineStr">
         <is>
-          <t>More related Persons</t>
+          <t>Related Persons</t>
         </is>
       </c>
       <c r="D60" s="1" t="inlineStr">
         <is>
-          <t>Mehr Personen</t>
+          <t>Verknüpfte Personen</t>
         </is>
       </c>
       <c r="E60" s="1" t="inlineStr">
@@ -1913,17 +1913,17 @@
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
-          <t>eth.placePage.topics</t>
+          <t>eth.personCard.headingMore</t>
         </is>
       </c>
       <c r="C61" s="1" t="inlineStr">
         <is>
-          <t>Topics in ETH swisscovery</t>
+          <t>More related Persons</t>
         </is>
       </c>
       <c r="D61" s="1" t="inlineStr">
         <is>
-          <t>Geografisches Schlagwort in ETH swisscovery</t>
+          <t>Mehr Personen</t>
         </is>
       </c>
       <c r="E61" s="1" t="inlineStr">
@@ -1943,17 +1943,17 @@
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
-          <t>eth.placePage.ethorama</t>
+          <t>eth.placePage.topics</t>
         </is>
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
-          <t>Documents in ETHorama</t>
+          <t>Topics in ETH swisscovery</t>
         </is>
       </c>
       <c r="D62" s="1" t="inlineStr">
         <is>
-          <t>Dokumente in ETHorama</t>
+          <t>Geografisches Schlagwort in ETH swisscovery</t>
         </is>
       </c>
       <c r="E62" s="1" t="inlineStr">
@@ -1973,17 +1973,17 @@
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
-          <t>eth.placePage.ethoramaTopics</t>
+          <t>eth.placePage.ethorama</t>
         </is>
       </c>
       <c r="C63" s="1" t="inlineStr">
         <is>
-          <t>ETHorama thematic collections</t>
+          <t>Documents in ETHorama</t>
         </is>
       </c>
       <c r="D63" s="1" t="inlineStr">
         <is>
-          <t>ETHorama Themensammlungen</t>
+          <t>Dokumente in ETHorama</t>
         </is>
       </c>
       <c r="E63" s="1" t="inlineStr">
@@ -2003,17 +2003,17 @@
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t>eth.placePage.ethoramaRoutes</t>
+          <t>eth.placePage.ethoramaTopics</t>
         </is>
       </c>
       <c r="C64" s="1" t="inlineStr">
         <is>
-          <t>ETHorama historical travels</t>
+          <t>ETHorama thematic collections</t>
         </is>
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t>ETHorama Historische Reisen</t>
+          <t>ETHorama Themensammlungen</t>
         </is>
       </c>
       <c r="E64" s="1" t="inlineStr">
@@ -2033,17 +2033,17 @@
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
-          <t>eth.placePage.wikidata</t>
+          <t>eth.placePage.ethoramaRoutes</t>
         </is>
       </c>
       <c r="C65" s="1" t="inlineStr">
         <is>
-          <t>Links from Wikidata</t>
+          <t>ETHorama historical travels</t>
         </is>
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>Links from Wikidata</t>
+          <t>ETHorama Historische Reisen</t>
         </is>
       </c>
       <c r="E65" s="1" t="inlineStr">
@@ -2063,17 +2063,17 @@
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
-          <t>eth.placePage.maps</t>
+          <t>eth.placePage.wikidata</t>
         </is>
       </c>
       <c r="C66" s="1" t="inlineStr">
         <is>
-          <t>Historical maps</t>
+          <t>Links from Wikidata</t>
         </is>
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t>Historische Karten</t>
+          <t>Links from Wikidata</t>
         </is>
       </c>
       <c r="E66" s="1" t="inlineStr">
@@ -2093,17 +2093,17 @@
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>eth.placePage.mapsList</t>
+          <t>eth.placePage.maps</t>
         </is>
       </c>
       <c r="C67" s="1" t="inlineStr">
         <is>
-          <t>Historical maps as list</t>
+          <t>Historical maps</t>
         </is>
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t>Historische Karten als Liste</t>
+          <t>Historische Karten</t>
         </is>
       </c>
       <c r="E67" s="1" t="inlineStr">
@@ -2123,17 +2123,17 @@
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.searchVariants</t>
+          <t>eth.placePage.mapsList</t>
         </is>
       </c>
       <c r="C68" s="1" t="inlineStr">
         <is>
-          <t>Search variants in all data of the ETH Library</t>
+          <t>Historical maps as list</t>
         </is>
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t>Suchvarianten in allen Daten der ETH-Bibliothek</t>
+          <t>Historische Karten als Liste</t>
         </is>
       </c>
       <c r="E68" s="1" t="inlineStr">
@@ -2153,17 +2153,17 @@
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.results</t>
+          <t>eth.personPage.searchVariants</t>
         </is>
       </c>
       <c r="C69" s="1" t="inlineStr">
         <is>
-          <t>results</t>
+          <t>Search variants in all data of the ETH Library</t>
         </is>
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>Ergebnisse</t>
+          <t>Suchvarianten in allen Daten der ETH-Bibliothek</t>
         </is>
       </c>
       <c r="E69" s="1" t="inlineStr">
@@ -2183,17 +2183,17 @@
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.authorityLinking</t>
+          <t>eth.personPage.results</t>
         </is>
       </c>
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t>Authority data</t>
+          <t>results</t>
         </is>
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>Normdaten</t>
+          <t>Ergebnisse</t>
         </is>
       </c>
       <c r="E70" s="1" t="inlineStr">
@@ -2213,17 +2213,17 @@
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.researcherProfile</t>
+          <t>eth.personPage.authorityLinking</t>
         </is>
       </c>
       <c r="C71" s="1" t="inlineStr">
         <is>
-          <t>Researcher profiles</t>
+          <t>Authority data</t>
         </is>
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>Forscherprofile</t>
+          <t>Normdaten</t>
         </is>
       </c>
       <c r="E71" s="1" t="inlineStr">
@@ -2243,17 +2243,17 @@
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.archives</t>
+          <t>eth.personPage.researcherProfile</t>
         </is>
       </c>
       <c r="C72" s="1" t="inlineStr">
         <is>
-          <t>Archives</t>
+          <t>Researcher profiles</t>
         </is>
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t>Archive</t>
+          <t>Forscherprofile</t>
         </is>
       </c>
       <c r="E72" s="1" t="inlineStr">
@@ -2273,17 +2273,17 @@
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.metagrid</t>
+          <t>eth.personPage.archives</t>
         </is>
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t>Metagrid</t>
+          <t>Archives</t>
         </is>
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t>Metagrid</t>
+          <t>Archive</t>
         </is>
       </c>
       <c r="E73" s="1" t="inlineStr">
@@ -2303,17 +2303,17 @@
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.wikidata</t>
+          <t>eth.personPage.metagrid</t>
         </is>
       </c>
       <c r="C74" s="1" t="inlineStr">
         <is>
-          <t>Wikidata</t>
+          <t>Metagrid</t>
         </is>
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t>Wikidata</t>
+          <t>Metagrid</t>
         </is>
       </c>
       <c r="E74" s="1" t="inlineStr">
@@ -2333,17 +2333,17 @@
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.prometheus</t>
+          <t>eth.personPage.wikidata</t>
         </is>
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t>Prometheus</t>
+          <t>Wikidata</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t>Prometheus</t>
+          <t>Wikidata</t>
         </is>
       </c>
       <c r="E75" s="1" t="inlineStr">
@@ -2363,17 +2363,17 @@
       </c>
       <c r="B76" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.students</t>
+          <t>eth.personPage.prometheus</t>
         </is>
       </c>
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t>Students (Wikidata)</t>
+          <t>Prometheus</t>
         </is>
       </c>
       <c r="D76" s="1" t="inlineStr">
         <is>
-          <t>Studenten (Wikidata)</t>
+          <t>Prometheus</t>
         </is>
       </c>
       <c r="E76" s="1" t="inlineStr">
@@ -2393,17 +2393,17 @@
       </c>
       <c r="B77" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.teacher</t>
+          <t>eth.personPage.students</t>
         </is>
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t>Teachers (Wikidata)</t>
+          <t>Students (Wikidata)</t>
         </is>
       </c>
       <c r="D77" s="1" t="inlineStr">
         <is>
-          <t>Lehrer (Wikidata)</t>
+          <t>Studenten (Wikidata)</t>
         </is>
       </c>
       <c r="E77" s="1" t="inlineStr">
@@ -2423,17 +2423,17 @@
       </c>
       <c r="B78" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.relatedGnd</t>
+          <t>eth.personPage.teacher</t>
         </is>
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>Related persons from GND</t>
+          <t>Teachers (Wikidata)</t>
         </is>
       </c>
       <c r="D78" s="1" t="inlineStr">
         <is>
-          <t>Verbundene Personen nach GND</t>
+          <t>Lehrer (Wikidata)</t>
         </is>
       </c>
       <c r="E78" s="1" t="inlineStr">
@@ -2453,17 +2453,17 @@
       </c>
       <c r="B79" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.prometheusIntro1</t>
+          <t>eth.personPage.relatedGnd</t>
         </is>
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t>Links from the</t>
+          <t>Related persons from GND</t>
         </is>
       </c>
       <c r="D79" s="1" t="inlineStr">
         <is>
-          <t>Links vom</t>
+          <t>Verbundene Personen nach GND</t>
         </is>
       </c>
       <c r="E79" s="1" t="inlineStr">
@@ -2483,17 +2483,17 @@
       </c>
       <c r="B80" s="1" t="inlineStr">
         <is>
-          <t>slsp.offCampusWarning.41SLSP_ETH:ETH_NDE</t>
+          <t>eth.personPage.prometheusIntro1</t>
         </is>
       </c>
       <c r="C80" s="1" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Licensed electronic resources of ETH Library are accessible only within the network of ETH Zurich.&lt;br&gt;&lt;a target="_blank" ng-href="https://unlimited.ethz.ch/display/WWE/Use+of+electronic+media+the+ETH+Library" rel="noopener" class="md-primoExplore-theme" href="https://unlimited.ethz.ch/display/WWE/Use+of+electronic+media+the+ETH+Library"&gt;Information about using electronic resources&lt;/a&gt; &lt;/p&gt;</t>
+          <t>Links from the</t>
         </is>
       </c>
       <c r="D80" s="1" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Lizenzierte E-Ressourcen der ETH-Bibliothek sind über das ETH-Netzwerk oder VPN zugänglich.&lt;br&gt; &lt;a target="_blank" ng-href="https://unlimited.ethz.ch/display/WWE/Use+of+electronic+media+the+ETH+Library" rel="noopener" class="md-primoExplore-theme" href="https://unlimited.ethz.ch/display/WWE/Use+of+electronic+media+the+ETH+Library"&gt;Informationen zur Nutzung elektronischer Ressourcen&lt;/a&gt; &lt;/p&gt;</t>
+          <t>Links vom</t>
         </is>
       </c>
       <c r="E80" s="1" t="inlineStr">
@@ -2502,7 +2502,7 @@
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>46253.0</v>
+        <v>46058.0</v>
       </c>
     </row>
     <row r="81">
@@ -2513,17 +2513,17 @@
       </c>
       <c r="B81" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.prometheusIntro2</t>
+          <t>slsp.offCampusWarning.41SLSP_ETH:ETH_NDE</t>
         </is>
       </c>
       <c r="C81" s="1" t="inlineStr">
         <is>
-          <t>Aggregator of the</t>
+          <t>&lt;p&gt;Licensed electronic resources of ETH Library are accessible only within the network of ETH Zurich.&lt;br&gt;&lt;a target="_blank" ng-href="https://unlimited.ethz.ch/display/WWE/Use+of+electronic+media+the+ETH+Library" rel="noopener" class="md-primoExplore-theme" href="https://unlimited.ethz.ch/display/WWE/Use+of+electronic+media+the+ETH+Library"&gt;Information about using electronic resources&lt;/a&gt; &lt;/p&gt;</t>
         </is>
       </c>
       <c r="D81" s="1" t="inlineStr">
         <is>
-          <t>Aggregator des</t>
+          <t>&lt;p&gt;Lizenzierte E-Ressourcen der ETH-Bibliothek sind über das ETH-Netzwerk oder VPN zugänglich.&lt;br&gt; &lt;a target="_blank" ng-href="https://unlimited.ethz.ch/display/WWE/Use+of+electronic+media+the+ETH+Library" rel="noopener" class="md-primoExplore-theme" href="https://unlimited.ethz.ch/display/WWE/Use+of+electronic+media+the+ETH+Library"&gt;Informationen zur Nutzung elektronischer Ressourcen&lt;/a&gt; &lt;/p&gt;</t>
         </is>
       </c>
       <c r="E81" s="1" t="inlineStr">
@@ -2532,7 +2532,7 @@
         </is>
       </c>
       <c r="F81" s="2" t="n">
-        <v>46058.0</v>
+        <v>46253.0</v>
       </c>
     </row>
     <row r="82">
@@ -2543,17 +2543,17 @@
       </c>
       <c r="B82" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.prometheusIntro3</t>
+          <t>eth.personPage.prometheusIntro2</t>
         </is>
       </c>
       <c r="C82" s="1" t="inlineStr">
         <is>
-          <t>LMU Center for Digital Humanities</t>
+          <t>Aggregator of the</t>
         </is>
       </c>
       <c r="D82" s="1" t="inlineStr">
         <is>
-          <t>LMU Center for Digital Humanities</t>
+          <t>Aggregator des</t>
         </is>
       </c>
       <c r="E82" s="1" t="inlineStr">
@@ -2573,17 +2573,17 @@
       </c>
       <c r="B83" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.searchName</t>
+          <t>eth.personPage.prometheusIntro3</t>
         </is>
       </c>
       <c r="C83" s="1" t="inlineStr">
         <is>
-          <t>Search by name</t>
+          <t>LMU Center for Digital Humanities</t>
         </is>
       </c>
       <c r="D83" s="1" t="inlineStr">
         <is>
-          <t>Suche nach Namen</t>
+          <t>LMU Center for Digital Humanities</t>
         </is>
       </c>
       <c r="E83" s="1" t="inlineStr">
@@ -2603,17 +2603,17 @@
       </c>
       <c r="B84" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.searchGnd</t>
+          <t>eth.personPage.searchName</t>
         </is>
       </c>
       <c r="C84" s="1" t="inlineStr">
         <is>
-          <t>Search by GND ID</t>
+          <t>Search by name</t>
         </is>
       </c>
       <c r="D84" s="1" t="inlineStr">
         <is>
-          <t>Suche nach GND ID</t>
+          <t>Suche nach Namen</t>
         </is>
       </c>
       <c r="E84" s="1" t="inlineStr">
@@ -2633,17 +2633,17 @@
       </c>
       <c r="B85" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.searchGndBirth</t>
+          <t>eth.personPage.searchGnd</t>
         </is>
       </c>
       <c r="C85" s="1" t="inlineStr">
         <is>
-          <t>Search by name and (GND ID or birthyear)</t>
+          <t>Search by GND ID</t>
         </is>
       </c>
       <c r="D85" s="1" t="inlineStr">
         <is>
-          <t>Suche nach Name und (GND ID oder Geburtsjahr)</t>
+          <t>Suche nach GND ID</t>
         </is>
       </c>
       <c r="E85" s="1" t="inlineStr">
@@ -2663,17 +2663,17 @@
       </c>
       <c r="B86" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.born</t>
+          <t>eth.personPage.searchGndBirth</t>
         </is>
       </c>
       <c r="C86" s="1" t="inlineStr">
         <is>
-          <t>Born:</t>
+          <t>Search by name and (GND ID or birthyear)</t>
         </is>
       </c>
       <c r="D86" s="1" t="inlineStr">
         <is>
-          <t>Geboren:</t>
+          <t>Suche nach Name und (GND ID oder Geburtsjahr)</t>
         </is>
       </c>
       <c r="E86" s="1" t="inlineStr">
@@ -2693,17 +2693,17 @@
       </c>
       <c r="B87" s="1" t="inlineStr">
         <is>
-          <t>eth.personPage.prometheusAll</t>
+          <t>eth.personPage.born</t>
         </is>
       </c>
       <c r="C87" s="1" t="inlineStr">
         <is>
-          <t>All links from Prometheus</t>
+          <t>Born:</t>
         </is>
       </c>
       <c r="D87" s="1" t="inlineStr">
         <is>
-          <t>Alle Links von Prometheus</t>
+          <t>Geboren:</t>
         </is>
       </c>
       <c r="E87" s="1" t="inlineStr">
@@ -2723,17 +2723,17 @@
       </c>
       <c r="B88" s="1" t="inlineStr">
         <is>
-          <t>eth.provenienzEraraLink.erara</t>
+          <t>eth.personPage.prometheusAll</t>
         </is>
       </c>
       <c r="C88" s="1" t="inlineStr">
         <is>
-          <t>Source in e-rara</t>
+          <t>All links from Prometheus</t>
         </is>
       </c>
       <c r="D88" s="1" t="inlineStr">
         <is>
-          <t>Quelle in e-rara</t>
+          <t>Alle Links von Prometheus</t>
         </is>
       </c>
       <c r="E88" s="1" t="inlineStr">
@@ -2753,17 +2753,17 @@
       </c>
       <c r="B89" s="1" t="inlineStr">
         <is>
-          <t>eth.provenienzEraraLink.swisscovery</t>
+          <t>eth.provenienzEraraLink.erara</t>
         </is>
       </c>
       <c r="C89" s="1" t="inlineStr">
         <is>
-          <t>Details provenance mark</t>
+          <t>Source in e-rara</t>
         </is>
       </c>
       <c r="D89" s="1" t="inlineStr">
         <is>
-          <t>Details Provenienzvermerk</t>
+          <t>Quelle in e-rara</t>
         </is>
       </c>
       <c r="E89" s="1" t="inlineStr">
@@ -2783,17 +2783,17 @@
       </c>
       <c r="B90" s="1" t="inlineStr">
         <is>
-          <t>eth.bibNews.heading</t>
+          <t>eth.provenienzEraraLink.swisscovery</t>
         </is>
       </c>
       <c r="C90" s="1" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Details provenance mark</t>
         </is>
       </c>
       <c r="D90" s="1" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Details Provenienzvermerk</t>
         </is>
       </c>
       <c r="E90" s="1" t="inlineStr">
@@ -2813,17 +2813,17 @@
       </c>
       <c r="B91" s="1" t="inlineStr">
         <is>
-          <t>eth.gitHint.heading</t>
+          <t>eth.bibNews.heading</t>
         </is>
       </c>
       <c r="C91" s="1" t="inlineStr">
         <is>
-          <t>important information</t>
+          <t>News</t>
         </is>
       </c>
       <c r="D91" s="1" t="inlineStr">
         <is>
-          <t>Wichtiger Hinweis</t>
+          <t>News</t>
         </is>
       </c>
       <c r="E91" s="1" t="inlineStr">
@@ -2843,17 +2843,17 @@
       </c>
       <c r="B92" s="1" t="inlineStr">
         <is>
-          <t>eth.locationLink.website</t>
+          <t>eth.gitHint.heading</t>
         </is>
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t>Website</t>
+          <t>important information</t>
         </is>
       </c>
       <c r="D92" s="1" t="inlineStr">
         <is>
-          <t>Webseite</t>
+          <t>Wichtiger Hinweis</t>
         </is>
       </c>
       <c r="E92" s="1" t="inlineStr">
@@ -2873,17 +2873,17 @@
       </c>
       <c r="B93" s="1" t="inlineStr">
         <is>
-          <t>eth.rapidoEthmemberHint.text</t>
+          <t>eth.locationLink.website</t>
         </is>
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t>Please check in the upper ordering section if one of the libraries at ETH Zurich offers "Digitization" (free service).</t>
+          <t>Website</t>
         </is>
       </c>
       <c r="D93" s="1" t="inlineStr">
         <is>
-          <t>Überprüfen Sie bitte im oberen Bestellbereich, ob eine Bibliothek der ETH Zürich "Digitalisierung" anbietet (kostenloser Service).</t>
+          <t>Webseite</t>
         </is>
       </c>
       <c r="E93" s="1" t="inlineStr">
@@ -2892,7 +2892,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>46108.0</v>
+        <v>46058.0</v>
       </c>
     </row>
     <row r="94">
@@ -2903,17 +2903,17 @@
       </c>
       <c r="B94" s="1" t="inlineStr">
         <is>
-          <t>41SLSP_ETH:TMI_NDE.eth.composeNb.print</t>
+          <t>eth.rapidoEthmemberHint.text</t>
         </is>
       </c>
       <c r="C94" s="1" t="inlineStr">
         <is>
-          <t>Print item in TMI Research</t>
+          <t>Please check in the upper ordering section if one of the libraries at ETH Zurich offers "Digitization" (free service).</t>
         </is>
       </c>
       <c r="D94" s="1" t="inlineStr">
         <is>
-          <t>Print-Exemplar in TMI Research</t>
+          <t>Überprüfen Sie bitte im oberen Bestellbereich, ob eine Bibliothek der ETH Zürich "Digitalisierung" anbietet (kostenloser Service).</t>
         </is>
       </c>
       <c r="E94" s="1" t="inlineStr">
@@ -2922,7 +2922,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>46113.0</v>
+        <v>46108.0</v>
       </c>
     </row>
     <row r="95">
@@ -2933,26 +2933,26 @@
       </c>
       <c r="B95" s="1" t="inlineStr">
         <is>
-          <t>41SLSP_ETH:ETH_NDE.nde.landing.header</t>
+          <t>41SLSP_ETH:TMI_NDE.eth.composeNb.print</t>
         </is>
       </c>
       <c r="C95" s="1" t="inlineStr">
         <is>
-          <t>ETH swisscovery</t>
+          <t>Print item in TMI Research</t>
         </is>
       </c>
       <c r="D95" s="1" t="inlineStr">
         <is>
-          <t>ETH swisscovery</t>
+          <t>Print-Exemplar in TMI Research</t>
         </is>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>noemie.ammann@library.ethz.ch</t>
+          <t>bernd.uttenweiler@library.ethz.ch</t>
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>46261.0</v>
+        <v>46113.0</v>
       </c>
     </row>
     <row r="96">
@@ -2963,26 +2963,26 @@
       </c>
       <c r="B96" s="1" t="inlineStr">
         <is>
-          <t>slsp.topbarMessage.message.41SLSP_ETH:ETH_NDE</t>
+          <t>41SLSP_ETH:ETH_NDE.nde.landing.header</t>
         </is>
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>NOT_DEFINED</t>
+          <t>ETH swisscovery</t>
         </is>
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>NOT_DEFINED</t>
+          <t>ETH swisscovery</t>
         </is>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>bernd.uttenweiler@library.ethz.ch</t>
+          <t>noemie.ammann@library.ethz.ch</t>
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>46240.0</v>
+        <v>46261.0</v>
       </c>
     </row>
     <row r="97">
@@ -2993,17 +2993,17 @@
       </c>
       <c r="B97" s="1" t="inlineStr">
         <is>
-          <t>41SLSP_ETH:TMI_NDE.eth.composeNb.online</t>
+          <t>slsp.topbarMessage.message.41SLSP_ETH:ETH_NDE</t>
         </is>
       </c>
       <c r="C97" s="1" t="inlineStr">
         <is>
-          <t>Online item in TMI Research</t>
+          <t>NOT_DEFINED</t>
         </is>
       </c>
       <c r="D97" s="1" t="inlineStr">
         <is>
-          <t>Online-Exemplar in TMI Research</t>
+          <t>NOT_DEFINED</t>
         </is>
       </c>
       <c r="E97" s="1" t="inlineStr">
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="F97" s="2" t="n">
-        <v>46113.0</v>
+        <v>46240.0</v>
       </c>
     </row>
     <row r="98">
@@ -3023,17 +3023,17 @@
       </c>
       <c r="B98" s="1" t="inlineStr">
         <is>
-          <t>41SLSP_ETH:TMI_NDE.eth.logoSubline.subline</t>
+          <t>41SLSP_ETH:TMI_NDE.eth.composeNb.online</t>
         </is>
       </c>
       <c r="C98" s="1" t="inlineStr">
         <is>
-          <t>TMI Research</t>
+          <t>Online item in TMI Research</t>
         </is>
       </c>
       <c r="D98" s="1" t="inlineStr">
         <is>
-          <t>TMI Research</t>
+          <t>Online-Exemplar in TMI Research</t>
         </is>
       </c>
       <c r="E98" s="1" t="inlineStr">
@@ -3053,17 +3053,17 @@
       </c>
       <c r="B99" s="1" t="inlineStr">
         <is>
-          <t>eth.requestHint.request</t>
+          <t>41SLSP_ETH:TMI_NDE.eth.logoSubline.subline</t>
         </is>
       </c>
       <c r="C99" s="1" t="inlineStr">
         <is>
-          <t>Pickup on site: free of charge&lt;br&gt;Postal delivery: CHF 12.00 (free of charge to ETH institutional address)</t>
+          <t>TMI Research</t>
         </is>
       </c>
       <c r="D99" s="1" t="inlineStr">
         <is>
-          <t>Abholung vor Ort: kostenlos&lt;br&gt;Postversand: CHF 12.00 (kostenlos an ETH-Institutsadresse)</t>
+          <t>TMI Research</t>
         </is>
       </c>
       <c r="E99" s="1" t="inlineStr">
@@ -3072,7 +3072,7 @@
         </is>
       </c>
       <c r="F99" s="2" t="n">
-        <v>46141.0</v>
+        <v>46113.0</v>
       </c>
     </row>
     <row r="100">
@@ -3083,17 +3083,17 @@
       </c>
       <c r="B100" s="1" t="inlineStr">
         <is>
-          <t>slsp.getit.reservationText</t>
+          <t>eth.requestHint.request</t>
         </is>
       </c>
       <c r="C100" s="1" t="inlineStr">
         <is>
-          <t>Reserve</t>
+          <t>Pickup on site: free of charge&lt;br&gt;Postal delivery: CHF 12.00 (free of charge to ETH institutional address)</t>
         </is>
       </c>
       <c r="D100" s="1" t="inlineStr">
         <is>
-          <t>Reservieren</t>
+          <t>Abholung vor Ort: kostenlos&lt;br&gt;Postversand: CHF 12.00 (kostenlos an ETH-Institutsadresse)</t>
         </is>
       </c>
       <c r="E100" s="1" t="inlineStr">
@@ -3102,7 +3102,7 @@
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>46266.0</v>
+        <v>46141.0</v>
       </c>
     </row>
     <row r="101">
@@ -3203,17 +3203,17 @@
       </c>
       <c r="B104" s="1" t="inlineStr">
         <is>
-          <t>eth.requestHint.digitizationOtherLibrary</t>
+          <t>eth.provenance.linkText</t>
         </is>
       </c>
       <c r="C104" s="1" t="inlineStr">
         <is>
-          <t>Normal fee: CHF 5.00&lt;br&gt;Commercial clients: CHF 25.00</t>
+          <t xml:space="preserve">Provenance </t>
         </is>
       </c>
       <c r="D104" s="1" t="inlineStr">
         <is>
-          <t>Normale Gebühr: CHF 5.00&lt;br&gt;Kommerzielle Unternehmen: CHF 25.00</t>
+          <t xml:space="preserve">Provenance </t>
         </is>
       </c>
       <c r="E104" s="1" t="inlineStr">
@@ -3222,7 +3222,7 @@
         </is>
       </c>
       <c r="F104" s="2" t="n">
-        <v>46142.0</v>
+        <v>46317.0</v>
       </c>
     </row>
     <row r="105">
@@ -3233,17 +3233,17 @@
       </c>
       <c r="B105" s="1" t="inlineStr">
         <is>
-          <t>tmi.getit.tmhla</t>
+          <t>eth.requestHint.digitizationOtherLibrary</t>
         </is>
       </c>
       <c r="C105" s="1" t="inlineStr">
         <is>
-          <t>&lt;div&gt;       &lt;span&gt;Not loanable.&lt;/span&gt;   &lt;/div&gt;   &lt;div&gt;       &lt;span&gt;Can be used in the library of the Thomas Mann House by prior appointment. Please contact&lt;/span&gt;       &lt;a href="mailto:thomasmannhouse@vatmh.org?subject=Request about: {{callNumber}}"&gt;           &lt;span&gt;thomasmannhouse@vatmh.org&lt;/span&gt;       &lt;/a&gt;          &lt;/div&gt;</t>
+          <t>Normal fee: CHF 5.00&lt;br&gt;Commercial clients: CHF 25.00</t>
         </is>
       </c>
       <c r="D105" s="1" t="inlineStr">
         <is>
-          <t>&lt;div&gt;  &lt;span&gt;Nicht ausleihbar.&lt;/span&gt;   &lt;/div&gt;   &lt;div&gt;       &lt;span&gt;Benutzung nach vorheriger Anmeldung in der Bibliothek des Thomas-Mann-Hauses. Bitte kontaktieren Sie&lt;/span&gt;       &lt;a href="mailto:thomasmannhouse@vatmh.org?subject=Anfrage zu: {{callNumber}}"&gt;           &lt;span&gt;thomasmannhouse@vatmh.org&lt;/span&gt;       &lt;/a&gt;          &lt;/div&gt;</t>
+          <t>Normale Gebühr: CHF 5.00&lt;br&gt;Kommerzielle Unternehmen: CHF 25.00</t>
         </is>
       </c>
       <c r="E105" s="1" t="inlineStr">
@@ -3252,7 +3252,7 @@
         </is>
       </c>
       <c r="F105" s="2" t="n">
-        <v>46149.0</v>
+        <v>46142.0</v>
       </c>
     </row>
     <row r="106">
@@ -3263,17 +3263,17 @@
       </c>
       <c r="B106" s="1" t="inlineStr">
         <is>
-          <t>eth.requestHint.requestOtherLibrary</t>
+          <t>tmi.getit.tmhla</t>
         </is>
       </c>
       <c r="C106" s="1" t="inlineStr">
         <is>
-          <t>Pickup on site: free of charge&lt;br&gt;Postal delivery: CHF 12.00</t>
+          <t>&lt;div&gt;       &lt;span&gt;Not loanable.&lt;/span&gt;   &lt;/div&gt;   &lt;div&gt;       &lt;span&gt;Can be used in the library of the Thomas Mann House by prior appointment. Please contact&lt;/span&gt;       &lt;a href="mailto:thomasmannhouse@vatmh.org?subject=Request about: {{callNumber}}"&gt;           &lt;span&gt;thomasmannhouse@vatmh.org&lt;/span&gt;       &lt;/a&gt;          &lt;/div&gt;</t>
         </is>
       </c>
       <c r="D106" s="1" t="inlineStr">
         <is>
-          <t>Abholung vor Ort: kostenlos&lt;br&gt;Postversand: CHF 12.00</t>
+          <t>&lt;div&gt;  &lt;span&gt;Nicht ausleihbar.&lt;/span&gt;   &lt;/div&gt;   &lt;div&gt;       &lt;span&gt;Benutzung nach vorheriger Anmeldung in der Bibliothek des Thomas-Mann-Hauses. Bitte kontaktieren Sie&lt;/span&gt;       &lt;a href="mailto:thomasmannhouse@vatmh.org?subject=Anfrage zu: {{callNumber}}"&gt;           &lt;span&gt;thomasmannhouse@vatmh.org&lt;/span&gt;       &lt;/a&gt;          &lt;/div&gt;</t>
         </is>
       </c>
       <c r="E106" s="1" t="inlineStr">
@@ -3282,7 +3282,7 @@
         </is>
       </c>
       <c r="F106" s="2" t="n">
-        <v>46142.0</v>
+        <v>46149.0</v>
       </c>
     </row>
     <row r="107">
@@ -3293,17 +3293,17 @@
       </c>
       <c r="B107" s="1" t="inlineStr">
         <is>
-          <t>tmi.getit.luebeck</t>
+          <t>eth.requestHint.requestOtherLibrary</t>
         </is>
       </c>
       <c r="C107" s="1" t="inlineStr">
         <is>
-          <t>&lt;a target="_blank" href="https://archiv-buddenbrookhaus.luebeck.de/objekt_start.fau?prj=buddenbrookhaus&amp;dm={{dm}}&amp;ref={{id}}"&gt;         Detailed information in the online database of the Buddenbrookhaus     &lt;/a&gt;     &lt;div&gt;         &lt;span&gt;Not possible to order.&lt;/span&gt;     &lt;/div&gt;     &lt;div&gt;Digital copies can be requested from Buddenbrookhaus (                 &lt;a href="mailto:britta.dittmann@luebeck.de?subject=Request about: {{callNumber}}"&gt;Contact&lt;/a&gt; ).     &lt;/div&gt;</t>
+          <t>Pickup on site: free of charge&lt;br&gt;Postal delivery: CHF 12.00</t>
         </is>
       </c>
       <c r="D107" s="1" t="inlineStr">
         <is>
-          <t>&lt;a target="_blank" href="https://archiv-buddenbrookhaus.luebeck.de/objekt_start.fau?prj=buddenbrookhaus&amp;dm={{dm}}&amp;ref={{id}}"&gt;         Detailinformationen in der Online-Datenbank des Buddenbrookhauses     &lt;/a&gt;     &lt;div&gt;         &lt;span&gt;Keine Bestellung möglich.&lt;/span&gt;     &lt;/div&gt;     &lt;div&gt;Digitalisate können beim Buddenbrookhaus angefragt werden (                 &lt;a href="mailto:britta.dittmann@luebeck.de?subject=Anfrage zu: {{callNumber}}"&gt;Kontakt&lt;/a&gt; ).     &lt;/div&gt;</t>
+          <t>Abholung vor Ort: kostenlos&lt;br&gt;Postversand: CHF 12.00</t>
         </is>
       </c>
       <c r="E107" s="1" t="inlineStr">
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="F107" s="2" t="n">
-        <v>46149.0</v>
+        <v>46142.0</v>
       </c>
     </row>
     <row r="108">
@@ -3323,17 +3323,17 @@
       </c>
       <c r="B108" s="1" t="inlineStr">
         <is>
-          <t>tmi.viewit.monacensia</t>
+          <t>tmi.getit.luebeck</t>
         </is>
       </c>
       <c r="C108" s="1" t="inlineStr">
         <is>
-          <t>&lt;a target="_blank" rel="noopener" href="{{link}}"&gt;Detailed information in the Kalliope Union Catalog (metadata only) &lt;/a&gt; &lt;div&gt;No request possible.&lt;/div&gt; &lt;div&gt;     Archival materials can be viewed on site at the Monacensia im Hildebrandhaus (     &lt;a href="mailto:monacensia.literaturarchiv@muenchen.de?subject=Request digitized copy with signature: {{callNumber}}"&gt;       Contact     &lt;/a&gt; ). &lt;/div&gt;</t>
+          <t>&lt;a target="_blank" href="https://archiv-buddenbrookhaus.luebeck.de/objekt_start.fau?prj=buddenbrookhaus&amp;dm={{dm}}&amp;ref={{id}}"&gt;         Detailed information in the online database of the Buddenbrookhaus     &lt;/a&gt;     &lt;div&gt;         &lt;span&gt;Not possible to order.&lt;/span&gt;     &lt;/div&gt;     &lt;div&gt;Digital copies can be requested from Buddenbrookhaus (                 &lt;a href="mailto:britta.dittmann@luebeck.de?subject=Request about: {{callNumber}}"&gt;Contact&lt;/a&gt; ).     &lt;/div&gt;</t>
         </is>
       </c>
       <c r="D108" s="1" t="inlineStr">
         <is>
-          <t>&lt;a target="_blank" rel="noopener" href="{{link}}"&gt;     Detailinformationen in der Online-Datenbank der Monacensia im Hildebrandhaus (nur Metadaten) &lt;/a&gt; &lt;div&gt;Keine Bestellung möglich.&lt;/div&gt; &lt;div&gt;     Archivalien können vor Ort in der Monacensia im Hildebrandhaus eingesehen werden (     &lt;a href="mailto:monacensia.literaturarchiv@muenchen.de?subject=Anfrage Digitalisat mit Signatur "{{callNumber}}""&gt;       Kontakt     &lt;/a&gt; ). &lt;/div&gt;</t>
+          <t>&lt;a target="_blank" href="https://archiv-buddenbrookhaus.luebeck.de/objekt_start.fau?prj=buddenbrookhaus&amp;dm={{dm}}&amp;ref={{id}}"&gt;         Detailinformationen in der Online-Datenbank des Buddenbrookhauses     &lt;/a&gt;     &lt;div&gt;         &lt;span&gt;Keine Bestellung möglich.&lt;/span&gt;     &lt;/div&gt;     &lt;div&gt;Digitalisate können beim Buddenbrookhaus angefragt werden (                 &lt;a href="mailto:britta.dittmann@luebeck.de?subject=Anfrage zu: {{callNumber}}"&gt;Kontakt&lt;/a&gt; ).     &lt;/div&gt;</t>
         </is>
       </c>
       <c r="E108" s="1" t="inlineStr">
@@ -3342,7 +3342,7 @@
         </is>
       </c>
       <c r="F108" s="2" t="n">
-        <v>46155.0</v>
+        <v>46149.0</v>
       </c>
     </row>
     <row r="109">
@@ -3353,17 +3353,17 @@
       </c>
       <c r="B109" s="1" t="inlineStr">
         <is>
-          <t>tmi.viewit.monacensia.heading</t>
+          <t>tmi.viewit.monacensia</t>
         </is>
       </c>
       <c r="C109" s="1" t="inlineStr">
         <is>
-          <t>Access</t>
+          <t>&lt;a target="_blank" rel="noopener" href="{{link}}"&gt;Detailed information in the Kalliope Union Catalog (metadata only) &lt;/a&gt; &lt;div&gt;No request possible.&lt;/div&gt; &lt;div&gt;     Archival materials can be viewed on site at the Monacensia im Hildebrandhaus (     &lt;a href="mailto:monacensia.literaturarchiv@muenchen.de?subject=Request digitized copy with signature: {{callNumber}}"&gt;       Contact     &lt;/a&gt; ). &lt;/div&gt;</t>
         </is>
       </c>
       <c r="D109" s="1" t="inlineStr">
         <is>
-          <t>Zugang</t>
+          <t>&lt;a target="_blank" rel="noopener" href="{{link}}"&gt;     Detailinformationen in der Online-Datenbank der Monacensia im Hildebrandhaus (nur Metadaten) &lt;/a&gt; &lt;div&gt;Keine Bestellung möglich.&lt;/div&gt; &lt;div&gt;     Archivalien können vor Ort in der Monacensia im Hildebrandhaus eingesehen werden (     &lt;a href="mailto:monacensia.literaturarchiv@muenchen.de?subject=Anfrage Digitalisat mit Signatur "{{callNumber}}""&gt;       Kontakt     &lt;/a&gt; ). &lt;/div&gt;</t>
         </is>
       </c>
       <c r="E109" s="1" t="inlineStr">
@@ -3383,17 +3383,17 @@
       </c>
       <c r="B110" s="1" t="inlineStr">
         <is>
-          <t>41SLSP_ETH:TMI_NDE.nde.landing.header</t>
+          <t>tmi.viewit.monacensia.heading</t>
         </is>
       </c>
       <c r="C110" s="1" t="inlineStr">
         <is>
-          <t>NOT_DEFINED</t>
+          <t>Access</t>
         </is>
       </c>
       <c r="D110" s="1" t="inlineStr">
         <is>
-          <t>NOT_DEFINED</t>
+          <t>Zugang</t>
         </is>
       </c>
       <c r="E110" s="1" t="inlineStr">
@@ -3402,7 +3402,7 @@
         </is>
       </c>
       <c r="F110" s="2" t="n">
-        <v>46164.0</v>
+        <v>46155.0</v>
       </c>
     </row>
     <row r="111">
@@ -3413,17 +3413,17 @@
       </c>
       <c r="B111" s="1" t="inlineStr">
         <is>
-          <t>eth.onlineProblem.mail</t>
+          <t>41SLSP_ETH:TMI_NDE.nde.landing.header</t>
         </is>
       </c>
       <c r="C111" s="1" t="inlineStr">
         <is>
-          <t>almakb@library.ethz.ch</t>
+          <t>NOT_DEFINED</t>
         </is>
       </c>
       <c r="D111" s="1" t="inlineStr">
         <is>
-          <t>almakb@library.ethz.ch</t>
+          <t>NOT_DEFINED</t>
         </is>
       </c>
       <c r="E111" s="1" t="inlineStr">
@@ -3432,7 +3432,7 @@
         </is>
       </c>
       <c r="F111" s="2" t="n">
-        <v>46169.0</v>
+        <v>46164.0</v>
       </c>
     </row>
     <row r="112">
@@ -3443,17 +3443,17 @@
       </c>
       <c r="B112" s="1" t="inlineStr">
         <is>
-          <t>tmi.topbarMessage.message</t>
+          <t>eth.onlineProblem.mail</t>
         </is>
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t>TMI EN:✨das und das momentan nicht möglich.  &lt;a href="https://library.ethz.ch/recherchieren-und-nutzen/research-assistant.html" target="_blank"&gt;Mehr erfahren&lt;/a&gt;</t>
+          <t>almakb@library.ethz.ch</t>
         </is>
       </c>
       <c r="D112" s="1" t="inlineStr">
         <is>
-          <t>TMI DE:✨das und das  nicht möglich.  &lt;a href="https://library.ethz.ch/recherchieren-und-nutzen/research-assistant.html" target="_blank"&gt;Mehr erfahren&lt;/a&gt;</t>
+          <t>almakb@library.ethz.ch</t>
         </is>
       </c>
       <c r="E112" s="1" t="inlineStr">
@@ -3462,7 +3462,7 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>46178.0</v>
+        <v>46169.0</v>
       </c>
     </row>
     <row r="113">
@@ -3473,17 +3473,17 @@
       </c>
       <c r="B113" s="1" t="inlineStr">
         <is>
-          <t>tmi.topbarMessage.heading</t>
+          <t>tmi.topbarMessage.message</t>
         </is>
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t>Important information</t>
+          <t>NOT_DEFINED</t>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
         <is>
-          <t>Wichtiger Hinweis</t>
+          <t>NOT_DEFINED</t>
         </is>
       </c>
       <c r="E113" s="1" t="inlineStr">
@@ -3492,7 +3492,7 @@
         </is>
       </c>
       <c r="F113" s="2" t="n">
-        <v>46178.0</v>
+        <v>46297.0</v>
       </c>
     </row>
     <row r="114">
@@ -3503,17 +3503,17 @@
       </c>
       <c r="B114" s="1" t="inlineStr">
         <is>
-          <t>tmi.composeErara.print</t>
+          <t>tmi.topbarMessage.heading</t>
         </is>
       </c>
       <c r="C114" s="1" t="inlineStr">
         <is>
-          <t>Print item in in ETH swisscovery</t>
+          <t>Important information</t>
         </is>
       </c>
       <c r="D114" s="1" t="inlineStr">
         <is>
-          <t>Print-Exemplar in TMI Research</t>
+          <t>Wichtiger Hinweis</t>
         </is>
       </c>
       <c r="E114" s="1" t="inlineStr">
@@ -3522,7 +3522,7 @@
         </is>
       </c>
       <c r="F114" s="2" t="n">
-        <v>46190.0</v>
+        <v>46178.0</v>
       </c>
     </row>
     <row r="115">
@@ -3533,17 +3533,17 @@
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>tmi.composeErara.online</t>
+          <t>tmi.composeErara.print</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>Online item in in ETH swisscovery</t>
+          <t>Print item in in ETH swisscovery</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>Online-Exemplar in TMI Research</t>
+          <t>Print-Exemplar in TMI Research</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
@@ -3555,8 +3555,38 @@
         <v>46190.0</v>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B116" s="1" t="inlineStr">
+        <is>
+          <t>tmi.composeErara.online</t>
+        </is>
+      </c>
+      <c r="C116" s="1" t="inlineStr">
+        <is>
+          <t>Online item in in ETH swisscovery</t>
+        </is>
+      </c>
+      <c r="D116" s="1" t="inlineStr">
+        <is>
+          <t>Online-Exemplar in TMI Research</t>
+        </is>
+      </c>
+      <c r="E116" s="1" t="inlineStr">
+        <is>
+          <t>bernd.uttenweiler@library.ethz.ch</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="n">
+        <v>46190.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F115"/>
+  <autoFilter ref="A1:F116"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>